<commit_message>
inventario att e montagem att
</commit_message>
<xml_diff>
--- a/INVENTARIO DE PECAS/inventario 2 mercado livre.xlsx
+++ b/INVENTARIO DE PECAS/inventario 2 mercado livre.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/573a85c25c05273f/RAFAEL VIDAL/EMPRESAS/ADITIV/DESENVOLVIMENTO/IMPRESSORA ADITIV/inventario/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nicholas\Desktop\Desenvolvimento_de_Impressora-3D-FFF-Open_Source-RepRap-_para_Odontologia_Digital\INVENTARIO DE PECAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="157" documentId="8_{F943354A-8C55-4439-B5C3-65D309E18260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B403480F-8EDC-4DBE-B940-FC74BB39FC56}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEC8832F-5836-4517-9D0B-88644F43187A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="98">
   <si>
     <t>Parafuso M3 10mm (allen)</t>
   </si>
@@ -325,6 +327,36 @@
   </si>
   <si>
     <t>EIXOS (h7 com espessura de cromo MAIOR QUE 0.15mm preferencialmente)</t>
+  </si>
+  <si>
+    <t>Sensor Indutivo M12 4mm Npn Na 3 Fios 5v Lj12a3-4-z/bx-5v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porca M5 </t>
+  </si>
+  <si>
+    <t>Parafuso M5  20mm</t>
+  </si>
+  <si>
+    <t>Parafuso M5 45mm</t>
+  </si>
+  <si>
+    <t>Parafuso M3 18 mm (allen)</t>
+  </si>
+  <si>
+    <t>Parafuso M5  30mm</t>
+  </si>
+  <si>
+    <t>Parafuso M3 15mm (allen)</t>
+  </si>
+  <si>
+    <t>Macal 12mm</t>
+  </si>
+  <si>
+    <t>Stop eixo y 8mm</t>
+  </si>
+  <si>
+    <t>Parafuso m4 CABEÇA CHATA 30mm</t>
   </si>
 </sst>
 </file>
@@ -462,10 +494,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2211,4 +2239,563 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D976A38-AFE1-4842-8215-8B96A1D93984}">
+  <dimension ref="A2:B90"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="85.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>82</v>
+      </c>
+      <c r="B47">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>26</v>
+      </c>
+      <c r="B50">
+        <f>2</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>83</v>
+      </c>
+      <c r="B51">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>75</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>27</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>30</v>
+      </c>
+      <c r="B54">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>28</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>76</v>
+      </c>
+      <c r="B56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>77</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>84</v>
+      </c>
+      <c r="B62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>63</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>55</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>31</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>73</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>66</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>36</v>
+      </c>
+      <c r="B74">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B76">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>46</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>65</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A83" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualização das instruções de montagem
</commit_message>
<xml_diff>
--- a/INVENTARIO DE PECAS/inventario 2 mercado livre.xlsx
+++ b/INVENTARIO DE PECAS/inventario 2 mercado livre.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nicholas\Desktop\Desenvolvimento_de_Impressora-3D-FFF-Open_Source-RepRap-_para_Odontologia_Digital\INVENTARIO DE PECAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEC8832F-5836-4517-9D0B-88644F43187A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74E10ED6-7AE2-4220-835A-6092A271680B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Planilha2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="99">
   <si>
     <t>Parafuso M3 10mm (allen)</t>
   </si>
@@ -357,6 +356,9 @@
   </si>
   <si>
     <t>Parafuso m4 CABEÇA CHATA 30mm</t>
+  </si>
+  <si>
+    <t>Parafuso M3 10mm CABEÇA CHATA</t>
   </si>
 </sst>
 </file>
@@ -2243,7 +2245,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D976A38-AFE1-4842-8215-8B96A1D93984}">
-  <dimension ref="A2:B90"/>
+  <dimension ref="A2:B91"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="85.5546875" customWidth="1"/>
@@ -2277,71 +2279,71 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B6">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="B10">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B12">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -2349,7 +2351,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>7</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -2357,228 +2359,228 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B16">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>93</v>
       </c>
-      <c r="B17">
+      <c r="B18">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20">
-        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>69</v>
       </c>
-      <c r="B21">
+      <c r="B22">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24">
-        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25">
-        <v>63</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26">
-        <v>22</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>89</v>
       </c>
-      <c r="B27">
+      <c r="B28">
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31">
-        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>35</v>
       </c>
-      <c r="B32">
+      <c r="B33">
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37">
-        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B38">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>96</v>
       </c>
-      <c r="B41">
+      <c r="B42">
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>24</v>
-      </c>
-      <c r="B44">
-        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B46">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B47">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="B48">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B50">
-        <f>2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="B51">
-        <v>6</v>
+        <f>2</f>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B53">
         <v>1</v>
@@ -2586,23 +2588,23 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B54">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="B56">
         <v>2</v>
@@ -2610,7 +2612,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>41</v>
+        <v>76</v>
       </c>
       <c r="B57">
         <v>2</v>
@@ -2618,64 +2620,64 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>77</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>84</v>
       </c>
-      <c r="B62">
+      <c r="B63">
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="6" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>63</v>
-      </c>
-      <c r="B66">
-        <v>1</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>55</v>
+        <v>63</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>55</v>
       </c>
-      <c r="B68">
-        <v>1</v>
-      </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B69">
         <v>1</v>
@@ -2683,7 +2685,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="B70">
         <v>1</v>
@@ -2691,20 +2693,20 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>74</v>
+        <v>31</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>73</v>
-      </c>
-      <c r="B72">
-        <v>1</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B73">
         <v>1</v>
@@ -2712,86 +2714,94 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="B74">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="B75">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="B76">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B77">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
+        <v>46</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>65</v>
-      </c>
-      <c r="B81">
-        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
+        <v>65</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A83" s="6" t="s">
+    <row r="84" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>